<commit_message>
feat: simplify learning episodes and preserve local attempts
</commit_message>
<xml_diff>
--- a/docs/concept-note-model.xlsx
+++ b/docs/concept-note-model.xlsx
@@ -619,7 +619,7 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner's own net income gain, as a share of the wage bill</t>
+          <t xml:space="preserve">Owner's own net income gain, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B20" s="4">
@@ -639,7 +639,7 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tax paid, as a share of the wage bill</t>
+          <t xml:space="preserve">Tax paid, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B21" s="4">
@@ -679,7 +679,7 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Local supplier income gain, as a share of the wage bill</t>
+          <t xml:space="preserve">Local supplier income gain, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B23" s="4">
@@ -1411,7 +1411,7 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wage bill, year 1</t>
+          <t xml:space="preserve">Worker income gain, year 1</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -1449,7 +1449,7 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">PV of wages</t>
+          <t xml:space="preserve">PV of worker income gains</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">The original reading. A fixed wage bill for a fixed period, nothing else.</t>
+          <t xml:space="preserve">The original reading. A fixed worker income-gain base for a fixed period, nothing else.</t>
         </is>
       </c>
     </row>
@@ -2447,73 +2447,73 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Annual income gain, non-transformational funded firm, USD</t>
+          <t xml:space="preserve">One-off build: portal, backend, AI judge, USD</t>
         </is>
       </c>
       <c r="B10" s="9">
-        <v>200</v>
+        <v>40000</v>
       </c>
       <c r="C10" s="9">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="D10" s="9">
-        <v>1.647</v>
+        <v>1.206</v>
       </c>
       <c r="E10" s="9">
-        <v>2.274</v>
+        <v>1.961</v>
       </c>
       <c r="F10" s="9">
-        <v>0.627</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displacement share — transformational firm</t>
+          <t xml:space="preserve">Annual income gain, non-transformational funded firm, USD</t>
         </is>
       </c>
       <c r="B11" s="9">
-        <v>0.4</v>
+        <v>200</v>
       </c>
       <c r="C11" s="9">
-        <v>0.05</v>
+        <v>700</v>
       </c>
       <c r="D11" s="9">
-        <v>1.595</v>
+        <v>1.647</v>
       </c>
       <c r="E11" s="9">
-        <v>2.107</v>
+        <v>2.274</v>
       </c>
       <c r="F11" s="9">
-        <v>0.512</v>
+        <v>0.627</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Local supplier income gain, as a share of the wage bill</t>
+          <t xml:space="preserve">Displacement share — transformational firm</t>
         </is>
       </c>
       <c r="B12" s="9">
-        <v>0.0</v>
+        <v>0.4</v>
       </c>
       <c r="C12" s="9">
-        <v>0.6</v>
+        <v>0.05</v>
       </c>
       <c r="D12" s="9">
-        <v>1.764</v>
+        <v>1.595</v>
       </c>
       <c r="E12" s="9">
-        <v>2.157</v>
+        <v>2.107</v>
       </c>
       <c r="F12" s="9">
-        <v>0.393</v>
+        <v>0.512</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner's own net income gain, as a share of the wage bill</t>
+          <t xml:space="preserve">Local supplier income gain, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B13" s="9">
@@ -2523,10 +2523,10 @@
         <v>0.6</v>
       </c>
       <c r="D13" s="9">
-        <v>1.731</v>
+        <v>1.764</v>
       </c>
       <c r="E13" s="9">
-        <v>2.124</v>
+        <v>2.157</v>
       </c>
       <c r="F13" s="9">
         <v>0.393</v>
@@ -2535,45 +2535,45 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recruitment cost per stage-0 start, USD</t>
+          <t xml:space="preserve">Owner's own net income gain, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B14" s="9">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="C14" s="9">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D14" s="9">
-        <v>1.718</v>
+        <v>1.731</v>
       </c>
       <c r="E14" s="9">
-        <v>2.109</v>
+        <v>2.124</v>
       </c>
       <c r="F14" s="9">
-        <v>0.391</v>
+        <v>0.393</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-off build: portal, backend, AI judge, USD</t>
+          <t xml:space="preserve">Recruitment cost per stage-0 start, USD</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <v>40000</v>
+        <v>5.0</v>
       </c>
       <c r="C15" s="9">
-        <v>15000</v>
+        <v>0.5</v>
       </c>
       <c r="D15" s="9">
-        <v>1.206</v>
+        <v>1.718</v>
       </c>
       <c r="E15" s="9">
-        <v>1.589</v>
+        <v>2.109</v>
       </c>
       <c r="F15" s="9">
-        <v>0.383</v>
+        <v>0.391</v>
       </c>
     </row>
     <row r="16">
@@ -2623,7 +2623,7 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tax paid, as a share of the wage bill</t>
+          <t xml:space="preserve">Tax paid, as a share of the worker income-gain base</t>
         </is>
       </c>
       <c r="B18" s="9">

</xml_diff>